<commit_message>
Added shame and exception dots to Discipline calendar
</commit_message>
<xml_diff>
--- a/Discipline/log.xlsx
+++ b/Discipline/log.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/876302c705ef890c/Documents/Website/Discipline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8F447EA2-AACC-4DB2-9706-D81718E4AFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{8F447EA2-AACC-4DB2-9706-D81718E4AFAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD1D5B3F-5EE3-4219-9AE4-5BA3D31CC577}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{522D815B-684E-4EC2-944D-228EE840B693}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -70,6 +70,18 @@
   </si>
   <si>
     <t>Climbing</t>
+  </si>
+  <si>
+    <t>Cleaning</t>
+  </si>
+  <si>
+    <t>LEGOing</t>
+  </si>
+  <si>
+    <t>Exceptional</t>
+  </si>
+  <si>
+    <t>Started log!</t>
   </si>
 </sst>
 </file>
@@ -125,9 +137,13 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{485D08B5-C08E-47FF-90E4-D0B139507F03}" name="Table1" displayName="Table1" ref="A1:C6" totalsRowShown="0">
-  <autoFilter ref="A1:C6" xr:uid="{485D08B5-C08E-47FF-90E4-D0B139507F03}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{485D08B5-C08E-47FF-90E4-D0B139507F03}" name="Table1" displayName="Table1" ref="A1:C15" totalsRowShown="0">
+  <autoFilter ref="A1:C15" xr:uid="{485D08B5-C08E-47FF-90E4-D0B139507F03}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{E26583C2-7705-4D42-98F1-A49733304A32}" name="Date"/>
     <tableColumn id="2" xr3:uid="{0240263F-2091-4E0E-98A9-3FF029B2D662}" name="Category"/>
@@ -454,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1407F29B-327C-41B1-8CB9-E5906D8333F9}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
@@ -522,10 +538,78 @@
         <v>46042</v>
       </c>
       <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>46042</v>
+      </c>
+      <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C7" t="s">
         <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>46043</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>46044</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>46044</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>46044</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
@@ -538,9 +622,9 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CF37EDC6-95EE-4C15-8E08-2E60D45926CC}">
           <x14:formula1>
-            <xm:f>Sheet2!$A$1:$A$3</xm:f>
+            <xm:f>Sheet2!$A$1:$A$4</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B6</xm:sqref>
+          <xm:sqref>B2:B15</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -550,7 +634,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{90408C74-5679-4472-B78E-65FB4ACE4686}">
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
@@ -568,6 +652,11 @@
         <v>5</v>
       </c>
     </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>